<commit_message>
:t-rex: run with filtered data => plots ("F70" version)
</commit_message>
<xml_diff>
--- a/data/derived_data/3_CommunityComposition/Dataset_1/ps_16S_rare_expe_D1_otu_table.xlsx
+++ b/data/derived_data/3_CommunityComposition/Dataset_1/ps_16S_rare_expe_D1_otu_table.xlsx
@@ -12,14 +12,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="84">
   <si>
     <t xml:space="preserve"/>
   </si>
   <si>
-    <t xml:space="preserve">MS_004</t>
-  </si>
-  <si>
     <t xml:space="preserve">MS_008</t>
   </si>
   <si>
@@ -213,15 +210,6 @@
   </si>
   <si>
     <t xml:space="preserve">MS_173</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MS_261</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MS_262</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MS_264</t>
   </si>
   <si>
     <t xml:space="preserve">MS_266</t>
@@ -821,40 +809,28 @@
       <c r="BT1" t="s">
         <v>71</v>
       </c>
-      <c r="BU1" t="s">
-        <v>72</v>
-      </c>
-      <c r="BV1" t="s">
-        <v>73</v>
-      </c>
-      <c r="BW1" t="s">
-        <v>74</v>
-      </c>
-      <c r="BX1" t="s">
-        <v>75</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B2" t="n">
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="G2" t="n">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -1049,99 +1025,87 @@
         <v>0</v>
       </c>
       <c r="BT2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BU2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BV2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BW2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BX2" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>231</v>
+      </c>
+      <c r="E3" t="n">
+        <v>258</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" t="n">
+        <v>1</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V3" t="n">
+        <v>5</v>
+      </c>
+      <c r="W3" t="n">
+        <v>7</v>
+      </c>
+      <c r="X3" t="n">
+        <v>24</v>
+      </c>
+      <c r="Y3" t="n">
         <v>26</v>
       </c>
-      <c r="D3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" t="n">
-        <v>231</v>
-      </c>
-      <c r="F3" t="n">
-        <v>258</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>0</v>
-      </c>
-      <c r="R3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S3" t="n">
-        <v>0</v>
-      </c>
-      <c r="T3" t="n">
-        <v>1</v>
-      </c>
-      <c r="U3" t="n">
-        <v>0</v>
-      </c>
-      <c r="V3" t="n">
-        <v>0</v>
-      </c>
-      <c r="W3" t="n">
-        <v>5</v>
-      </c>
-      <c r="X3" t="n">
-        <v>7</v>
-      </c>
-      <c r="Y3" t="n">
-        <v>24</v>
-      </c>
       <c r="Z3" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="AA3" t="n">
         <v>0</v>
@@ -1279,24 +1243,12 @@
         <v>0</v>
       </c>
       <c r="BT3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BU3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BV3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BW3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BX3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B4" t="n">
         <v>0</v>
@@ -1323,10 +1275,10 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="K4" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -1347,151 +1299,151 @@
         <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>0</v>
+        <v>149</v>
       </c>
       <c r="S4" t="n">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="T4" t="n">
-        <v>153</v>
+        <v>7</v>
       </c>
       <c r="U4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="W4" t="n">
         <v>1</v>
       </c>
       <c r="X4" t="n">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="Y4" t="n">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="Z4" t="n">
-        <v>49</v>
+        <v>128</v>
       </c>
       <c r="AA4" t="n">
-        <v>128</v>
+        <v>116</v>
       </c>
       <c r="AB4" t="n">
+        <v>69</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>55</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>175</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>95</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>101</v>
+      </c>
+      <c r="AM4" t="n">
+        <v>75</v>
+      </c>
+      <c r="AN4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV4" t="n">
+        <v>72</v>
+      </c>
+      <c r="AW4" t="n">
+        <v>69</v>
+      </c>
+      <c r="AX4" t="n">
+        <v>79</v>
+      </c>
+      <c r="AY4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD4" t="n">
+        <v>102</v>
+      </c>
+      <c r="BE4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ4" t="n">
+        <v>76</v>
+      </c>
+      <c r="BK4" t="n">
         <v>116</v>
       </c>
-      <c r="AC4" t="n">
-        <v>69</v>
-      </c>
-      <c r="AD4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF4" t="n">
-        <v>55</v>
-      </c>
-      <c r="AG4" t="n">
-        <v>175</v>
-      </c>
-      <c r="AH4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI4" t="n">
-        <v>95</v>
-      </c>
-      <c r="AJ4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM4" t="n">
-        <v>101</v>
-      </c>
-      <c r="AN4" t="n">
-        <v>75</v>
-      </c>
-      <c r="AO4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW4" t="n">
-        <v>72</v>
-      </c>
-      <c r="AX4" t="n">
-        <v>69</v>
-      </c>
-      <c r="AY4" t="n">
-        <v>79</v>
-      </c>
-      <c r="AZ4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE4" t="n">
-        <v>102</v>
-      </c>
-      <c r="BF4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BH4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BI4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BJ4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BK4" t="n">
-        <v>76</v>
-      </c>
       <c r="BL4" t="n">
-        <v>116</v>
+        <v>0</v>
       </c>
       <c r="BM4" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="BN4" t="n">
-        <v>71</v>
+        <v>0</v>
       </c>
       <c r="BO4" t="n">
         <v>0</v>
@@ -1500,42 +1452,30 @@
         <v>0</v>
       </c>
       <c r="BQ4" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="BR4" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="BS4" t="n">
         <v>0</v>
       </c>
       <c r="BT4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BU4" t="n">
-        <v>50</v>
-      </c>
-      <c r="BV4" t="n">
-        <v>8</v>
-      </c>
-      <c r="BW4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BX4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B5" t="n">
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>83</v>
       </c>
       <c r="D5" t="n">
-        <v>83</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -1739,39 +1679,27 @@
         <v>0</v>
       </c>
       <c r="BT5" t="n">
-        <v>0</v>
-      </c>
-      <c r="BU5" t="n">
-        <v>0</v>
-      </c>
-      <c r="BV5" t="n">
-        <v>0</v>
-      </c>
-      <c r="BW5" t="n">
-        <v>0</v>
-      </c>
-      <c r="BX5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="C6" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D6" t="n">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F6" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -1795,43 +1723,43 @@
         <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" t="n">
         <v>1</v>
       </c>
-      <c r="R6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T6" t="n">
-        <v>0</v>
-      </c>
       <c r="U6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" t="n">
         <v>1</v>
       </c>
-      <c r="V6" t="n">
-        <v>0</v>
-      </c>
-      <c r="W6" t="n">
-        <v>0</v>
-      </c>
-      <c r="X6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y6" t="n">
-        <v>0</v>
-      </c>
       <c r="Z6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA6" t="n">
         <v>0</v>
@@ -1969,24 +1897,12 @@
         <v>0</v>
       </c>
       <c r="BT6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BU6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BV6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BW6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BX6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B7" t="n">
         <v>0</v>
@@ -1995,13 +1911,13 @@
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E7" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F7" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -2199,42 +2115,30 @@
         <v>0</v>
       </c>
       <c r="BT7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BU7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BV7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BW7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BX7" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>2942</v>
       </c>
       <c r="C8" t="n">
-        <v>2942</v>
+        <v>2876</v>
       </c>
       <c r="D8" t="n">
-        <v>2876</v>
+        <v>2756</v>
       </c>
       <c r="E8" t="n">
-        <v>2756</v>
+        <v>2559</v>
       </c>
       <c r="F8" t="n">
-        <v>2559</v>
+        <v>2959</v>
       </c>
       <c r="G8" t="n">
-        <v>2959</v>
+        <v>3000</v>
       </c>
       <c r="H8" t="n">
         <v>3000</v>
@@ -2243,210 +2147,198 @@
         <v>3000</v>
       </c>
       <c r="J8" t="n">
+        <v>2606</v>
+      </c>
+      <c r="K8" t="n">
+        <v>2808</v>
+      </c>
+      <c r="L8" t="n">
+        <v>2572</v>
+      </c>
+      <c r="M8" t="n">
+        <v>519</v>
+      </c>
+      <c r="N8" t="n">
+        <v>2727</v>
+      </c>
+      <c r="O8" t="n">
+        <v>2564</v>
+      </c>
+      <c r="P8" t="n">
+        <v>2602</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>2714</v>
+      </c>
+      <c r="R8" t="n">
+        <v>1830</v>
+      </c>
+      <c r="S8" t="n">
+        <v>1859</v>
+      </c>
+      <c r="T8" t="n">
+        <v>1831</v>
+      </c>
+      <c r="U8" t="n">
+        <v>1800</v>
+      </c>
+      <c r="V8" t="n">
+        <v>1745</v>
+      </c>
+      <c r="W8" t="n">
+        <v>1884</v>
+      </c>
+      <c r="X8" t="n">
+        <v>1312</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>1763</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>1016</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>979</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>444</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>776</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI8" t="n">
+        <v>706</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>320</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP8" t="n">
+        <v>789</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS8" t="n">
+        <v>39</v>
+      </c>
+      <c r="AT8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV8" t="n">
+        <v>235</v>
+      </c>
+      <c r="AW8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO8" t="n">
+        <v>1230</v>
+      </c>
+      <c r="BP8" t="n">
         <v>3000</v>
       </c>
-      <c r="K8" t="n">
-        <v>2606</v>
-      </c>
-      <c r="L8" t="n">
-        <v>2808</v>
-      </c>
-      <c r="M8" t="n">
-        <v>2572</v>
-      </c>
-      <c r="N8" t="n">
-        <v>519</v>
-      </c>
-      <c r="O8" t="n">
-        <v>2727</v>
-      </c>
-      <c r="P8" t="n">
-        <v>2564</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>2602</v>
-      </c>
-      <c r="R8" t="n">
-        <v>2714</v>
-      </c>
-      <c r="S8" t="n">
-        <v>1830</v>
-      </c>
-      <c r="T8" t="n">
-        <v>1859</v>
-      </c>
-      <c r="U8" t="n">
-        <v>1831</v>
-      </c>
-      <c r="V8" t="n">
-        <v>1800</v>
-      </c>
-      <c r="W8" t="n">
-        <v>1745</v>
-      </c>
-      <c r="X8" t="n">
-        <v>1884</v>
-      </c>
-      <c r="Y8" t="n">
-        <v>1312</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>1763</v>
-      </c>
-      <c r="AA8" t="n">
-        <v>1016</v>
-      </c>
-      <c r="AB8" t="n">
-        <v>979</v>
-      </c>
-      <c r="AC8" t="n">
-        <v>444</v>
-      </c>
-      <c r="AD8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE8" t="n">
-        <v>776</v>
-      </c>
-      <c r="AF8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ8" t="n">
-        <v>706</v>
-      </c>
-      <c r="AK8" t="n">
-        <v>320</v>
-      </c>
-      <c r="AL8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ8" t="n">
-        <v>789</v>
-      </c>
-      <c r="AR8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT8" t="n">
-        <v>39</v>
-      </c>
-      <c r="AU8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW8" t="n">
-        <v>235</v>
-      </c>
-      <c r="AX8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BH8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BI8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BJ8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BK8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BL8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BN8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BO8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BP8" t="n">
-        <v>0</v>
-      </c>
       <c r="BQ8" t="n">
-        <v>0</v>
+        <v>2238</v>
       </c>
       <c r="BR8" t="n">
-        <v>0</v>
+        <v>2562</v>
       </c>
       <c r="BS8" t="n">
-        <v>1230</v>
+        <v>3000</v>
       </c>
       <c r="BT8" t="n">
-        <v>3000</v>
-      </c>
-      <c r="BU8" t="n">
-        <v>2238</v>
-      </c>
-      <c r="BV8" t="n">
-        <v>2562</v>
-      </c>
-      <c r="BW8" t="n">
-        <v>3000</v>
-      </c>
-      <c r="BX8" t="n">
         <v>2559</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B9" t="n">
         <v>0</v>
@@ -2458,10 +2350,10 @@
         <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>151</v>
       </c>
       <c r="F9" t="n">
-        <v>151</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -2659,24 +2551,12 @@
         <v>0</v>
       </c>
       <c r="BT9" t="n">
-        <v>0</v>
-      </c>
-      <c r="BU9" t="n">
-        <v>0</v>
-      </c>
-      <c r="BV9" t="n">
-        <v>0</v>
-      </c>
-      <c r="BW9" t="n">
-        <v>0</v>
-      </c>
-      <c r="BX9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B10" t="n">
         <v>0</v>
@@ -2703,10 +2583,10 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>217</v>
       </c>
       <c r="K10" t="n">
-        <v>217</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
@@ -2715,118 +2595,118 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>0</v>
+        <v>268</v>
       </c>
       <c r="O10" t="n">
-        <v>268</v>
+        <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>0</v>
+        <v>397</v>
       </c>
       <c r="Q10" t="n">
-        <v>397</v>
+        <v>286</v>
       </c>
       <c r="R10" t="n">
-        <v>286</v>
+        <v>58</v>
       </c>
       <c r="S10" t="n">
-        <v>58</v>
+        <v>120</v>
       </c>
       <c r="T10" t="n">
-        <v>120</v>
+        <v>1161</v>
       </c>
       <c r="U10" t="n">
-        <v>1161</v>
+        <v>1194</v>
       </c>
       <c r="V10" t="n">
-        <v>1194</v>
+        <v>1245</v>
       </c>
       <c r="W10" t="n">
-        <v>1245</v>
+        <v>1108</v>
       </c>
       <c r="X10" t="n">
-        <v>1108</v>
+        <v>7</v>
       </c>
       <c r="Y10" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="Z10" t="n">
-        <v>0</v>
+        <v>1581</v>
       </c>
       <c r="AA10" t="n">
-        <v>1581</v>
+        <v>1605</v>
       </c>
       <c r="AB10" t="n">
-        <v>1605</v>
+        <v>2394</v>
       </c>
       <c r="AC10" t="n">
-        <v>2394</v>
+        <v>3000</v>
       </c>
       <c r="AD10" t="n">
+        <v>2224</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>669</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG10" t="n">
         <v>3000</v>
       </c>
-      <c r="AE10" t="n">
-        <v>2224</v>
-      </c>
-      <c r="AF10" t="n">
-        <v>669</v>
-      </c>
-      <c r="AG10" t="n">
-        <v>0</v>
-      </c>
       <c r="AH10" t="n">
+        <v>2404</v>
+      </c>
+      <c r="AI10" t="n">
+        <v>2294</v>
+      </c>
+      <c r="AJ10" t="n">
+        <v>2680</v>
+      </c>
+      <c r="AK10" t="n">
         <v>3000</v>
       </c>
-      <c r="AI10" t="n">
-        <v>2404</v>
-      </c>
-      <c r="AJ10" t="n">
-        <v>2294</v>
-      </c>
-      <c r="AK10" t="n">
-        <v>2680</v>
-      </c>
       <c r="AL10" t="n">
+        <v>1821</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>676</v>
+      </c>
+      <c r="AN10" t="n">
         <v>3000</v>
-      </c>
-      <c r="AM10" t="n">
-        <v>1821</v>
-      </c>
-      <c r="AN10" t="n">
-        <v>676</v>
       </c>
       <c r="AO10" t="n">
         <v>3000</v>
       </c>
       <c r="AP10" t="n">
+        <v>2211</v>
+      </c>
+      <c r="AQ10" t="n">
         <v>3000</v>
-      </c>
-      <c r="AQ10" t="n">
-        <v>2211</v>
       </c>
       <c r="AR10" t="n">
         <v>3000</v>
       </c>
       <c r="AS10" t="n">
+        <v>2961</v>
+      </c>
+      <c r="AT10" t="n">
         <v>3000</v>
-      </c>
-      <c r="AT10" t="n">
-        <v>2961</v>
       </c>
       <c r="AU10" t="n">
         <v>3000</v>
       </c>
       <c r="AV10" t="n">
+        <v>2530</v>
+      </c>
+      <c r="AW10" t="n">
+        <v>676</v>
+      </c>
+      <c r="AX10" t="n">
+        <v>483</v>
+      </c>
+      <c r="AY10" t="n">
         <v>3000</v>
-      </c>
-      <c r="AW10" t="n">
-        <v>2530</v>
-      </c>
-      <c r="AX10" t="n">
-        <v>676</v>
-      </c>
-      <c r="AY10" t="n">
-        <v>483</v>
       </c>
       <c r="AZ10" t="n">
         <v>3000</v>
@@ -2841,10 +2721,10 @@
         <v>3000</v>
       </c>
       <c r="BD10" t="n">
+        <v>900</v>
+      </c>
+      <c r="BE10" t="n">
         <v>3000</v>
-      </c>
-      <c r="BE10" t="n">
-        <v>900</v>
       </c>
       <c r="BF10" t="n">
         <v>3000</v>
@@ -2859,57 +2739,45 @@
         <v>3000</v>
       </c>
       <c r="BJ10" t="n">
+        <v>798</v>
+      </c>
+      <c r="BK10" t="n">
+        <v>1894</v>
+      </c>
+      <c r="BL10" t="n">
+        <v>2870</v>
+      </c>
+      <c r="BM10" t="n">
+        <v>2640</v>
+      </c>
+      <c r="BN10" t="n">
         <v>3000</v>
       </c>
-      <c r="BK10" t="n">
-        <v>798</v>
-      </c>
-      <c r="BL10" t="n">
-        <v>1894</v>
-      </c>
-      <c r="BM10" t="n">
-        <v>2870</v>
-      </c>
-      <c r="BN10" t="n">
-        <v>2640</v>
-      </c>
       <c r="BO10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="BP10" t="n">
         <v>0</v>
       </c>
       <c r="BQ10" t="n">
-        <v>0</v>
+        <v>517</v>
       </c>
       <c r="BR10" t="n">
-        <v>0</v>
+        <v>401</v>
       </c>
       <c r="BS10" t="n">
         <v>0</v>
       </c>
       <c r="BT10" t="n">
-        <v>0</v>
-      </c>
-      <c r="BU10" t="n">
-        <v>517</v>
-      </c>
-      <c r="BV10" t="n">
-        <v>401</v>
-      </c>
-      <c r="BW10" t="n">
-        <v>0</v>
-      </c>
-      <c r="BX10" t="n">
         <v>404</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B11" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="C11" t="n">
         <v>0</v>
@@ -2933,82 +2801,82 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>0</v>
+        <v>146</v>
       </c>
       <c r="K11" t="n">
-        <v>146</v>
+        <v>192</v>
       </c>
       <c r="L11" t="n">
-        <v>192</v>
+        <v>428</v>
       </c>
       <c r="M11" t="n">
-        <v>428</v>
+        <v>2481</v>
       </c>
       <c r="N11" t="n">
-        <v>2481</v>
+        <v>0</v>
       </c>
       <c r="O11" t="n">
-        <v>0</v>
+        <v>436</v>
       </c>
       <c r="P11" t="n">
-        <v>436</v>
+        <v>0</v>
       </c>
       <c r="Q11" t="n">
         <v>0</v>
       </c>
       <c r="R11" t="n">
-        <v>0</v>
+        <v>963</v>
       </c>
       <c r="S11" t="n">
-        <v>963</v>
+        <v>867</v>
       </c>
       <c r="T11" t="n">
-        <v>867</v>
+        <v>0</v>
       </c>
       <c r="U11" t="n">
         <v>0</v>
       </c>
       <c r="V11" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="W11" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="X11" t="n">
-        <v>0</v>
+        <v>1630</v>
       </c>
       <c r="Y11" t="n">
-        <v>1630</v>
+        <v>1161</v>
       </c>
       <c r="Z11" t="n">
-        <v>1161</v>
+        <v>55</v>
       </c>
       <c r="AA11" t="n">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="AB11" t="n">
-        <v>59</v>
+        <v>92</v>
       </c>
       <c r="AC11" t="n">
-        <v>92</v>
+        <v>0</v>
       </c>
       <c r="AD11" t="n">
         <v>0</v>
       </c>
       <c r="AE11" t="n">
-        <v>0</v>
+        <v>494</v>
       </c>
       <c r="AF11" t="n">
-        <v>494</v>
+        <v>234</v>
       </c>
       <c r="AG11" t="n">
-        <v>234</v>
+        <v>0</v>
       </c>
       <c r="AH11" t="n">
-        <v>0</v>
+        <v>501</v>
       </c>
       <c r="AI11" t="n">
-        <v>501</v>
+        <v>0</v>
       </c>
       <c r="AJ11" t="n">
         <v>0</v>
@@ -3020,10 +2888,10 @@
         <v>0</v>
       </c>
       <c r="AM11" t="n">
-        <v>0</v>
+        <v>197</v>
       </c>
       <c r="AN11" t="n">
-        <v>197</v>
+        <v>0</v>
       </c>
       <c r="AO11" t="n">
         <v>0</v>
@@ -3071,10 +2939,10 @@
         <v>0</v>
       </c>
       <c r="BD11" t="n">
-        <v>0</v>
+        <v>1998</v>
       </c>
       <c r="BE11" t="n">
-        <v>1998</v>
+        <v>0</v>
       </c>
       <c r="BF11" t="n">
         <v>0</v>
@@ -3104,39 +2972,27 @@
         <v>0</v>
       </c>
       <c r="BO11" t="n">
-        <v>0</v>
+        <v>1770</v>
       </c>
       <c r="BP11" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="BQ11" t="n">
-        <v>3000</v>
+        <v>195</v>
       </c>
       <c r="BR11" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="BS11" t="n">
-        <v>1770</v>
+        <v>0</v>
       </c>
       <c r="BT11" t="n">
-        <v>0</v>
-      </c>
-      <c r="BU11" t="n">
-        <v>195</v>
-      </c>
-      <c r="BV11" t="n">
-        <v>0</v>
-      </c>
-      <c r="BW11" t="n">
-        <v>0</v>
-      </c>
-      <c r="BX11" t="n">
         <v>37</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B12" t="n">
         <v>0</v>
@@ -3148,10 +3004,10 @@
         <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F12" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
@@ -3349,24 +3205,12 @@
         <v>0</v>
       </c>
       <c r="BT12" t="n">
-        <v>0</v>
-      </c>
-      <c r="BU12" t="n">
-        <v>0</v>
-      </c>
-      <c r="BV12" t="n">
-        <v>0</v>
-      </c>
-      <c r="BW12" t="n">
-        <v>0</v>
-      </c>
-      <c r="BX12" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B13" t="n">
         <v>0</v>
@@ -3441,28 +3285,28 @@
         <v>0</v>
       </c>
       <c r="Z13" t="n">
-        <v>0</v>
+        <v>220</v>
       </c>
       <c r="AA13" t="n">
-        <v>220</v>
+        <v>241</v>
       </c>
       <c r="AB13" t="n">
-        <v>241</v>
+        <v>1</v>
       </c>
       <c r="AC13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD13" t="n">
         <v>0</v>
       </c>
       <c r="AE13" t="n">
-        <v>0</v>
+        <v>1782</v>
       </c>
       <c r="AF13" t="n">
-        <v>1782</v>
+        <v>2591</v>
       </c>
       <c r="AG13" t="n">
-        <v>2591</v>
+        <v>0</v>
       </c>
       <c r="AH13" t="n">
         <v>0</v>
@@ -3477,13 +3321,13 @@
         <v>0</v>
       </c>
       <c r="AL13" t="n">
-        <v>0</v>
+        <v>1078</v>
       </c>
       <c r="AM13" t="n">
-        <v>1078</v>
+        <v>2052</v>
       </c>
       <c r="AN13" t="n">
-        <v>2052</v>
+        <v>0</v>
       </c>
       <c r="AO13" t="n">
         <v>0</v>
@@ -3507,16 +3351,16 @@
         <v>0</v>
       </c>
       <c r="AV13" t="n">
-        <v>0</v>
+        <v>163</v>
       </c>
       <c r="AW13" t="n">
-        <v>163</v>
+        <v>2255</v>
       </c>
       <c r="AX13" t="n">
-        <v>2255</v>
+        <v>2438</v>
       </c>
       <c r="AY13" t="n">
-        <v>2438</v>
+        <v>0</v>
       </c>
       <c r="AZ13" t="n">
         <v>0</v>
@@ -3549,19 +3393,19 @@
         <v>0</v>
       </c>
       <c r="BJ13" t="n">
-        <v>0</v>
+        <v>2126</v>
       </c>
       <c r="BK13" t="n">
-        <v>2126</v>
+        <v>990</v>
       </c>
       <c r="BL13" t="n">
-        <v>990</v>
+        <v>130</v>
       </c>
       <c r="BM13" t="n">
-        <v>130</v>
+        <v>289</v>
       </c>
       <c r="BN13" t="n">
-        <v>289</v>
+        <v>0</v>
       </c>
       <c r="BO13" t="n">
         <v>0</v>
@@ -3573,24 +3417,12 @@
         <v>0</v>
       </c>
       <c r="BR13" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="BS13" t="n">
         <v>0</v>
       </c>
       <c r="BT13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BU13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BV13" t="n">
-        <v>29</v>
-      </c>
-      <c r="BW13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BX13" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
:pizza: include "Mothers_0days" for composition description + manually add "Cluster_66" ITS taxonomy
</commit_message>
<xml_diff>
--- a/data/derived_data/3_CommunityComposition/Dataset_1/ps_16S_rare_expe_D1_otu_table.xlsx
+++ b/data/derived_data/3_CommunityComposition/Dataset_1/ps_16S_rare_expe_D1_otu_table.xlsx
@@ -12,11 +12,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="88">
   <si>
     <t xml:space="preserve"/>
   </si>
   <si>
+    <t xml:space="preserve">MS_004</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_008</t>
   </si>
   <si>
@@ -210,6 +213,15 @@
   </si>
   <si>
     <t xml:space="preserve">MS_173</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_261</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_262</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_264</t>
   </si>
   <si>
     <t xml:space="preserve">MS_266</t>
@@ -809,29 +821,41 @@
       <c r="BT1" t="s">
         <v>71</v>
       </c>
+      <c r="BU1" t="s">
+        <v>72</v>
+      </c>
+      <c r="BV1" t="s">
+        <v>73</v>
+      </c>
+      <c r="BW1" t="s">
+        <v>74</v>
+      </c>
+      <c r="BX1" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B2" t="n">
         <v>0</v>
       </c>
       <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
         <v>2</v>
       </c>
-      <c r="D2" t="n">
-        <v>0</v>
-      </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
         <v>41</v>
       </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
       <c r="H2" t="n">
         <v>0</v>
       </c>
@@ -1025,28 +1049,40 @@
         <v>0</v>
       </c>
       <c r="BT2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX2" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="n">
         <v>26</v>
       </c>
-      <c r="C3" t="n">
-        <v>0</v>
-      </c>
       <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
         <v>231</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>258</v>
       </c>
-      <c r="F3" t="n">
-        <v>0</v>
-      </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
@@ -1084,29 +1120,29 @@
         <v>0</v>
       </c>
       <c r="S3" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" t="n">
         <v>1</v>
       </c>
-      <c r="T3" t="n">
-        <v>0</v>
-      </c>
       <c r="U3" t="n">
         <v>0</v>
       </c>
       <c r="V3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" t="n">
         <v>5</v>
       </c>
-      <c r="W3" t="n">
+      <c r="X3" t="n">
         <v>7</v>
       </c>
-      <c r="X3" t="n">
+      <c r="Y3" t="n">
         <v>24</v>
       </c>
-      <c r="Y3" t="n">
+      <c r="Z3" t="n">
         <v>26</v>
       </c>
-      <c r="Z3" t="n">
-        <v>0</v>
-      </c>
       <c r="AA3" t="n">
         <v>0</v>
       </c>
@@ -1243,12 +1279,24 @@
         <v>0</v>
       </c>
       <c r="BT3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="B4" t="n">
         <v>0</v>
@@ -1275,11 +1323,11 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
         <v>31</v>
       </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
       <c r="L4" t="n">
         <v>0</v>
       </c>
@@ -1299,59 +1347,59 @@
         <v>0</v>
       </c>
       <c r="R4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" t="n">
         <v>149</v>
       </c>
-      <c r="S4" t="n">
+      <c r="T4" t="n">
         <v>153</v>
       </c>
-      <c r="T4" t="n">
+      <c r="U4" t="n">
         <v>7</v>
       </c>
-      <c r="U4" t="n">
+      <c r="V4" t="n">
         <v>6</v>
-      </c>
-      <c r="V4" t="n">
-        <v>1</v>
       </c>
       <c r="W4" t="n">
         <v>1</v>
       </c>
       <c r="X4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y4" t="n">
         <v>27</v>
       </c>
-      <c r="Y4" t="n">
+      <c r="Z4" t="n">
         <v>49</v>
       </c>
-      <c r="Z4" t="n">
+      <c r="AA4" t="n">
         <v>128</v>
       </c>
-      <c r="AA4" t="n">
+      <c r="AB4" t="n">
         <v>116</v>
       </c>
-      <c r="AB4" t="n">
+      <c r="AC4" t="n">
         <v>69</v>
       </c>
-      <c r="AC4" t="n">
-        <v>0</v>
-      </c>
       <c r="AD4" t="n">
         <v>0</v>
       </c>
       <c r="AE4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF4" t="n">
         <v>55</v>
       </c>
-      <c r="AF4" t="n">
+      <c r="AG4" t="n">
         <v>175</v>
       </c>
-      <c r="AG4" t="n">
-        <v>0</v>
-      </c>
       <c r="AH4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI4" t="n">
         <v>95</v>
       </c>
-      <c r="AI4" t="n">
-        <v>0</v>
-      </c>
       <c r="AJ4" t="n">
         <v>0</v>
       </c>
@@ -1359,14 +1407,14 @@
         <v>0</v>
       </c>
       <c r="AL4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM4" t="n">
         <v>101</v>
       </c>
-      <c r="AM4" t="n">
+      <c r="AN4" t="n">
         <v>75</v>
       </c>
-      <c r="AN4" t="n">
-        <v>0</v>
-      </c>
       <c r="AO4" t="n">
         <v>0</v>
       </c>
@@ -1389,17 +1437,17 @@
         <v>0</v>
       </c>
       <c r="AV4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW4" t="n">
         <v>72</v>
       </c>
-      <c r="AW4" t="n">
+      <c r="AX4" t="n">
         <v>69</v>
       </c>
-      <c r="AX4" t="n">
+      <c r="AY4" t="n">
         <v>79</v>
       </c>
-      <c r="AY4" t="n">
-        <v>0</v>
-      </c>
       <c r="AZ4" t="n">
         <v>0</v>
       </c>
@@ -1413,11 +1461,11 @@
         <v>0</v>
       </c>
       <c r="BD4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE4" t="n">
         <v>102</v>
       </c>
-      <c r="BE4" t="n">
-        <v>0</v>
-      </c>
       <c r="BF4" t="n">
         <v>0</v>
       </c>
@@ -1431,20 +1479,20 @@
         <v>0</v>
       </c>
       <c r="BJ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK4" t="n">
         <v>76</v>
       </c>
-      <c r="BK4" t="n">
+      <c r="BL4" t="n">
         <v>116</v>
       </c>
-      <c r="BL4" t="n">
-        <v>0</v>
-      </c>
       <c r="BM4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN4" t="n">
         <v>71</v>
       </c>
-      <c r="BN4" t="n">
-        <v>0</v>
-      </c>
       <c r="BO4" t="n">
         <v>0</v>
       </c>
@@ -1452,31 +1500,43 @@
         <v>0</v>
       </c>
       <c r="BQ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU4" t="n">
         <v>50</v>
       </c>
-      <c r="BR4" t="n">
+      <c r="BV4" t="n">
         <v>8</v>
       </c>
-      <c r="BS4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BT4" t="n">
+      <c r="BW4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B5" t="n">
         <v>0</v>
       </c>
       <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
         <v>83</v>
       </c>
-      <c r="D5" t="n">
-        <v>0</v>
-      </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
@@ -1679,28 +1739,40 @@
         <v>0</v>
       </c>
       <c r="BT5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="n">
         <v>32</v>
       </c>
-      <c r="C6" t="n">
+      <c r="D6" t="n">
         <v>39</v>
       </c>
-      <c r="D6" t="n">
-        <v>0</v>
-      </c>
       <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
         <v>21</v>
       </c>
-      <c r="F6" t="n">
-        <v>0</v>
-      </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
@@ -1723,17 +1795,17 @@
         <v>0</v>
       </c>
       <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
         <v>5</v>
       </c>
-      <c r="O6" t="n">
-        <v>0</v>
-      </c>
       <c r="P6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="n">
         <v>1</v>
       </c>
-      <c r="Q6" t="n">
-        <v>0</v>
-      </c>
       <c r="R6" t="n">
         <v>0</v>
       </c>
@@ -1741,11 +1813,11 @@
         <v>0</v>
       </c>
       <c r="T6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" t="n">
         <v>1</v>
       </c>
-      <c r="U6" t="n">
-        <v>0</v>
-      </c>
       <c r="V6" t="n">
         <v>0</v>
       </c>
@@ -1756,11 +1828,11 @@
         <v>0</v>
       </c>
       <c r="Y6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z6" t="n">
         <v>1</v>
       </c>
-      <c r="Z6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA6" t="n">
         <v>0</v>
       </c>
@@ -1897,12 +1969,24 @@
         <v>0</v>
       </c>
       <c r="BT6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B7" t="n">
         <v>0</v>
@@ -1911,14 +1995,14 @@
         <v>0</v>
       </c>
       <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
         <v>13</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>9</v>
       </c>
-      <c r="F7" t="n">
-        <v>0</v>
-      </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
@@ -2115,30 +2199,42 @@
         <v>0</v>
       </c>
       <c r="BT7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX7" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="n">
         <v>2942</v>
       </c>
-      <c r="C8" t="n">
+      <c r="D8" t="n">
         <v>2876</v>
       </c>
-      <c r="D8" t="n">
+      <c r="E8" t="n">
         <v>2756</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>2559</v>
       </c>
-      <c r="F8" t="n">
+      <c r="G8" t="n">
         <v>2959</v>
-      </c>
-      <c r="G8" t="n">
-        <v>3000</v>
       </c>
       <c r="H8" t="n">
         <v>3000</v>
@@ -2147,71 +2243,71 @@
         <v>3000</v>
       </c>
       <c r="J8" t="n">
+        <v>3000</v>
+      </c>
+      <c r="K8" t="n">
         <v>2606</v>
       </c>
-      <c r="K8" t="n">
+      <c r="L8" t="n">
         <v>2808</v>
       </c>
-      <c r="L8" t="n">
+      <c r="M8" t="n">
         <v>2572</v>
       </c>
-      <c r="M8" t="n">
+      <c r="N8" t="n">
         <v>519</v>
       </c>
-      <c r="N8" t="n">
+      <c r="O8" t="n">
         <v>2727</v>
       </c>
-      <c r="O8" t="n">
+      <c r="P8" t="n">
         <v>2564</v>
       </c>
-      <c r="P8" t="n">
+      <c r="Q8" t="n">
         <v>2602</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="R8" t="n">
         <v>2714</v>
       </c>
-      <c r="R8" t="n">
+      <c r="S8" t="n">
         <v>1830</v>
       </c>
-      <c r="S8" t="n">
+      <c r="T8" t="n">
         <v>1859</v>
       </c>
-      <c r="T8" t="n">
+      <c r="U8" t="n">
         <v>1831</v>
       </c>
-      <c r="U8" t="n">
+      <c r="V8" t="n">
         <v>1800</v>
       </c>
-      <c r="V8" t="n">
+      <c r="W8" t="n">
         <v>1745</v>
       </c>
-      <c r="W8" t="n">
+      <c r="X8" t="n">
         <v>1884</v>
       </c>
-      <c r="X8" t="n">
+      <c r="Y8" t="n">
         <v>1312</v>
       </c>
-      <c r="Y8" t="n">
+      <c r="Z8" t="n">
         <v>1763</v>
       </c>
-      <c r="Z8" t="n">
+      <c r="AA8" t="n">
         <v>1016</v>
       </c>
-      <c r="AA8" t="n">
+      <c r="AB8" t="n">
         <v>979</v>
       </c>
-      <c r="AB8" t="n">
+      <c r="AC8" t="n">
         <v>444</v>
       </c>
-      <c r="AC8" t="n">
-        <v>0</v>
-      </c>
       <c r="AD8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE8" t="n">
         <v>776</v>
       </c>
-      <c r="AE8" t="n">
-        <v>0</v>
-      </c>
       <c r="AF8" t="n">
         <v>0</v>
       </c>
@@ -2222,14 +2318,14 @@
         <v>0</v>
       </c>
       <c r="AI8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ8" t="n">
         <v>706</v>
       </c>
-      <c r="AJ8" t="n">
+      <c r="AK8" t="n">
         <v>320</v>
       </c>
-      <c r="AK8" t="n">
-        <v>0</v>
-      </c>
       <c r="AL8" t="n">
         <v>0</v>
       </c>
@@ -2243,29 +2339,29 @@
         <v>0</v>
       </c>
       <c r="AP8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ8" t="n">
         <v>789</v>
       </c>
-      <c r="AQ8" t="n">
-        <v>0</v>
-      </c>
       <c r="AR8" t="n">
         <v>0</v>
       </c>
       <c r="AS8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT8" t="n">
         <v>39</v>
       </c>
-      <c r="AT8" t="n">
-        <v>0</v>
-      </c>
       <c r="AU8" t="n">
         <v>0</v>
       </c>
       <c r="AV8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW8" t="n">
         <v>235</v>
       </c>
-      <c r="AW8" t="n">
-        <v>0</v>
-      </c>
       <c r="AX8" t="n">
         <v>0</v>
       </c>
@@ -2318,27 +2414,39 @@
         <v>0</v>
       </c>
       <c r="BO8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS8" t="n">
         <v>1230</v>
       </c>
-      <c r="BP8" t="n">
+      <c r="BT8" t="n">
         <v>3000</v>
       </c>
-      <c r="BQ8" t="n">
+      <c r="BU8" t="n">
         <v>2238</v>
       </c>
-      <c r="BR8" t="n">
+      <c r="BV8" t="n">
         <v>2562</v>
       </c>
-      <c r="BS8" t="n">
+      <c r="BW8" t="n">
         <v>3000</v>
       </c>
-      <c r="BT8" t="n">
+      <c r="BX8" t="n">
         <v>2559</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B9" t="n">
         <v>0</v>
@@ -2350,11 +2458,11 @@
         <v>0</v>
       </c>
       <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
         <v>151</v>
       </c>
-      <c r="F9" t="n">
-        <v>0</v>
-      </c>
       <c r="G9" t="n">
         <v>0</v>
       </c>
@@ -2551,12 +2659,24 @@
         <v>0</v>
       </c>
       <c r="BT9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B10" t="n">
         <v>0</v>
@@ -2583,11 +2703,11 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
         <v>217</v>
       </c>
-      <c r="K10" t="n">
-        <v>0</v>
-      </c>
       <c r="L10" t="n">
         <v>0</v>
       </c>
@@ -2595,118 +2715,118 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="n">
         <v>268</v>
       </c>
-      <c r="O10" t="n">
-        <v>0</v>
-      </c>
       <c r="P10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="n">
         <v>397</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="R10" t="n">
         <v>286</v>
       </c>
-      <c r="R10" t="n">
+      <c r="S10" t="n">
         <v>58</v>
       </c>
-      <c r="S10" t="n">
+      <c r="T10" t="n">
         <v>120</v>
       </c>
-      <c r="T10" t="n">
+      <c r="U10" t="n">
         <v>1161</v>
       </c>
-      <c r="U10" t="n">
+      <c r="V10" t="n">
         <v>1194</v>
       </c>
-      <c r="V10" t="n">
+      <c r="W10" t="n">
         <v>1245</v>
       </c>
-      <c r="W10" t="n">
+      <c r="X10" t="n">
         <v>1108</v>
       </c>
-      <c r="X10" t="n">
+      <c r="Y10" t="n">
         <v>7</v>
       </c>
-      <c r="Y10" t="n">
-        <v>0</v>
-      </c>
       <c r="Z10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA10" t="n">
         <v>1581</v>
       </c>
-      <c r="AA10" t="n">
+      <c r="AB10" t="n">
         <v>1605</v>
       </c>
-      <c r="AB10" t="n">
+      <c r="AC10" t="n">
         <v>2394</v>
       </c>
-      <c r="AC10" t="n">
+      <c r="AD10" t="n">
         <v>3000</v>
       </c>
-      <c r="AD10" t="n">
+      <c r="AE10" t="n">
         <v>2224</v>
       </c>
-      <c r="AE10" t="n">
+      <c r="AF10" t="n">
         <v>669</v>
       </c>
-      <c r="AF10" t="n">
-        <v>0</v>
-      </c>
       <c r="AG10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH10" t="n">
         <v>3000</v>
       </c>
-      <c r="AH10" t="n">
+      <c r="AI10" t="n">
         <v>2404</v>
       </c>
-      <c r="AI10" t="n">
+      <c r="AJ10" t="n">
         <v>2294</v>
       </c>
-      <c r="AJ10" t="n">
+      <c r="AK10" t="n">
         <v>2680</v>
       </c>
-      <c r="AK10" t="n">
+      <c r="AL10" t="n">
         <v>3000</v>
       </c>
-      <c r="AL10" t="n">
+      <c r="AM10" t="n">
         <v>1821</v>
       </c>
-      <c r="AM10" t="n">
+      <c r="AN10" t="n">
         <v>676</v>
-      </c>
-      <c r="AN10" t="n">
-        <v>3000</v>
       </c>
       <c r="AO10" t="n">
         <v>3000</v>
       </c>
       <c r="AP10" t="n">
+        <v>3000</v>
+      </c>
+      <c r="AQ10" t="n">
         <v>2211</v>
-      </c>
-      <c r="AQ10" t="n">
-        <v>3000</v>
       </c>
       <c r="AR10" t="n">
         <v>3000</v>
       </c>
       <c r="AS10" t="n">
+        <v>3000</v>
+      </c>
+      <c r="AT10" t="n">
         <v>2961</v>
-      </c>
-      <c r="AT10" t="n">
-        <v>3000</v>
       </c>
       <c r="AU10" t="n">
         <v>3000</v>
       </c>
       <c r="AV10" t="n">
+        <v>3000</v>
+      </c>
+      <c r="AW10" t="n">
         <v>2530</v>
       </c>
-      <c r="AW10" t="n">
+      <c r="AX10" t="n">
         <v>676</v>
       </c>
-      <c r="AX10" t="n">
+      <c r="AY10" t="n">
         <v>483</v>
-      </c>
-      <c r="AY10" t="n">
-        <v>3000</v>
       </c>
       <c r="AZ10" t="n">
         <v>3000</v>
@@ -2721,10 +2841,10 @@
         <v>3000</v>
       </c>
       <c r="BD10" t="n">
+        <v>3000</v>
+      </c>
+      <c r="BE10" t="n">
         <v>900</v>
-      </c>
-      <c r="BE10" t="n">
-        <v>3000</v>
       </c>
       <c r="BF10" t="n">
         <v>3000</v>
@@ -2739,45 +2859,57 @@
         <v>3000</v>
       </c>
       <c r="BJ10" t="n">
+        <v>3000</v>
+      </c>
+      <c r="BK10" t="n">
         <v>798</v>
       </c>
-      <c r="BK10" t="n">
+      <c r="BL10" t="n">
         <v>1894</v>
       </c>
-      <c r="BL10" t="n">
+      <c r="BM10" t="n">
         <v>2870</v>
       </c>
-      <c r="BM10" t="n">
+      <c r="BN10" t="n">
         <v>2640</v>
       </c>
-      <c r="BN10" t="n">
+      <c r="BO10" t="n">
         <v>3000</v>
       </c>
-      <c r="BO10" t="n">
-        <v>0</v>
-      </c>
       <c r="BP10" t="n">
         <v>0</v>
       </c>
       <c r="BQ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU10" t="n">
         <v>517</v>
       </c>
-      <c r="BR10" t="n">
+      <c r="BV10" t="n">
         <v>401</v>
       </c>
-      <c r="BS10" t="n">
-        <v>0</v>
-      </c>
-      <c r="BT10" t="n">
+      <c r="BW10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX10" t="n">
         <v>404</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="C11" t="n">
         <v>0</v>
@@ -2801,83 +2933,83 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
         <v>146</v>
       </c>
-      <c r="K11" t="n">
+      <c r="L11" t="n">
         <v>192</v>
       </c>
-      <c r="L11" t="n">
+      <c r="M11" t="n">
         <v>428</v>
       </c>
-      <c r="M11" t="n">
+      <c r="N11" t="n">
         <v>2481</v>
       </c>
-      <c r="N11" t="n">
-        <v>0</v>
-      </c>
       <c r="O11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" t="n">
         <v>436</v>
       </c>
-      <c r="P11" t="n">
-        <v>0</v>
-      </c>
       <c r="Q11" t="n">
         <v>0</v>
       </c>
       <c r="R11" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" t="n">
         <v>963</v>
       </c>
-      <c r="S11" t="n">
+      <c r="T11" t="n">
         <v>867</v>
       </c>
-      <c r="T11" t="n">
-        <v>0</v>
-      </c>
       <c r="U11" t="n">
         <v>0</v>
       </c>
       <c r="V11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W11" t="n">
         <v>4</v>
       </c>
-      <c r="W11" t="n">
-        <v>0</v>
-      </c>
       <c r="X11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y11" t="n">
         <v>1630</v>
       </c>
-      <c r="Y11" t="n">
+      <c r="Z11" t="n">
         <v>1161</v>
       </c>
-      <c r="Z11" t="n">
+      <c r="AA11" t="n">
         <v>55</v>
       </c>
-      <c r="AA11" t="n">
+      <c r="AB11" t="n">
         <v>59</v>
       </c>
-      <c r="AB11" t="n">
+      <c r="AC11" t="n">
         <v>92</v>
       </c>
-      <c r="AC11" t="n">
-        <v>0</v>
-      </c>
       <c r="AD11" t="n">
         <v>0</v>
       </c>
       <c r="AE11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF11" t="n">
         <v>494</v>
       </c>
-      <c r="AF11" t="n">
+      <c r="AG11" t="n">
         <v>234</v>
       </c>
-      <c r="AG11" t="n">
-        <v>0</v>
-      </c>
       <c r="AH11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI11" t="n">
         <v>501</v>
       </c>
-      <c r="AI11" t="n">
-        <v>0</v>
-      </c>
       <c r="AJ11" t="n">
         <v>0</v>
       </c>
@@ -2888,11 +3020,11 @@
         <v>0</v>
       </c>
       <c r="AM11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN11" t="n">
         <v>197</v>
       </c>
-      <c r="AN11" t="n">
-        <v>0</v>
-      </c>
       <c r="AO11" t="n">
         <v>0</v>
       </c>
@@ -2939,11 +3071,11 @@
         <v>0</v>
       </c>
       <c r="BD11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE11" t="n">
         <v>1998</v>
       </c>
-      <c r="BE11" t="n">
-        <v>0</v>
-      </c>
       <c r="BF11" t="n">
         <v>0</v>
       </c>
@@ -2972,27 +3104,39 @@
         <v>0</v>
       </c>
       <c r="BO11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP11" t="n">
+        <v>3000</v>
+      </c>
+      <c r="BQ11" t="n">
+        <v>3000</v>
+      </c>
+      <c r="BR11" t="n">
+        <v>3000</v>
+      </c>
+      <c r="BS11" t="n">
         <v>1770</v>
       </c>
-      <c r="BP11" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ11" t="n">
+      <c r="BT11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU11" t="n">
         <v>195</v>
       </c>
-      <c r="BR11" t="n">
-        <v>0</v>
-      </c>
-      <c r="BS11" t="n">
-        <v>0</v>
-      </c>
-      <c r="BT11" t="n">
+      <c r="BV11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX11" t="n">
         <v>37</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B12" t="n">
         <v>0</v>
@@ -3004,11 +3148,11 @@
         <v>0</v>
       </c>
       <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
         <v>2</v>
       </c>
-      <c r="F12" t="n">
-        <v>0</v>
-      </c>
       <c r="G12" t="n">
         <v>0</v>
       </c>
@@ -3205,12 +3349,24 @@
         <v>0</v>
       </c>
       <c r="BT12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX12" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B13" t="n">
         <v>0</v>
@@ -3285,29 +3441,29 @@
         <v>0</v>
       </c>
       <c r="Z13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA13" t="n">
         <v>220</v>
       </c>
-      <c r="AA13" t="n">
+      <c r="AB13" t="n">
         <v>241</v>
       </c>
-      <c r="AB13" t="n">
+      <c r="AC13" t="n">
         <v>1</v>
       </c>
-      <c r="AC13" t="n">
-        <v>0</v>
-      </c>
       <c r="AD13" t="n">
         <v>0</v>
       </c>
       <c r="AE13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF13" t="n">
         <v>1782</v>
       </c>
-      <c r="AF13" t="n">
+      <c r="AG13" t="n">
         <v>2591</v>
       </c>
-      <c r="AG13" t="n">
-        <v>0</v>
-      </c>
       <c r="AH13" t="n">
         <v>0</v>
       </c>
@@ -3321,14 +3477,14 @@
         <v>0</v>
       </c>
       <c r="AL13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM13" t="n">
         <v>1078</v>
       </c>
-      <c r="AM13" t="n">
+      <c r="AN13" t="n">
         <v>2052</v>
       </c>
-      <c r="AN13" t="n">
-        <v>0</v>
-      </c>
       <c r="AO13" t="n">
         <v>0</v>
       </c>
@@ -3351,17 +3507,17 @@
         <v>0</v>
       </c>
       <c r="AV13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW13" t="n">
         <v>163</v>
       </c>
-      <c r="AW13" t="n">
+      <c r="AX13" t="n">
         <v>2255</v>
       </c>
-      <c r="AX13" t="n">
+      <c r="AY13" t="n">
         <v>2438</v>
       </c>
-      <c r="AY13" t="n">
-        <v>0</v>
-      </c>
       <c r="AZ13" t="n">
         <v>0</v>
       </c>
@@ -3393,20 +3549,20 @@
         <v>0</v>
       </c>
       <c r="BJ13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK13" t="n">
         <v>2126</v>
       </c>
-      <c r="BK13" t="n">
+      <c r="BL13" t="n">
         <v>990</v>
       </c>
-      <c r="BL13" t="n">
+      <c r="BM13" t="n">
         <v>130</v>
       </c>
-      <c r="BM13" t="n">
+      <c r="BN13" t="n">
         <v>289</v>
       </c>
-      <c r="BN13" t="n">
-        <v>0</v>
-      </c>
       <c r="BO13" t="n">
         <v>0</v>
       </c>
@@ -3417,12 +3573,24 @@
         <v>0</v>
       </c>
       <c r="BR13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV13" t="n">
         <v>29</v>
       </c>
-      <c r="BS13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BT13" t="n">
+      <c r="BW13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX13" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
:herb: compo bar plots with clean taxo & data filtered at prev >= 60 %
</commit_message>
<xml_diff>
--- a/data/derived_data/3_CommunityComposition/Dataset_1/ps_16S_rare_expe_D1_otu_table.xlsx
+++ b/data/derived_data/3_CommunityComposition/Dataset_1/ps_16S_rare_expe_D1_otu_table.xlsx
@@ -12,11 +12,17 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="114">
   <si>
     <t xml:space="preserve"/>
   </si>
   <si>
+    <t xml:space="preserve">MS_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_003</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_004</t>
   </si>
   <si>
@@ -41,12 +47,21 @@
     <t xml:space="preserve">MS_025</t>
   </si>
   <si>
+    <t xml:space="preserve">MS_026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_027</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_028</t>
   </si>
   <si>
     <t xml:space="preserve">MS_030</t>
   </si>
   <si>
+    <t xml:space="preserve">MS_032</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_035</t>
   </si>
   <si>
@@ -59,6 +74,9 @@
     <t xml:space="preserve">MS_038</t>
   </si>
   <si>
+    <t xml:space="preserve">MS_039</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_040</t>
   </si>
   <si>
@@ -80,6 +98,12 @@
     <t xml:space="preserve">MS_060</t>
   </si>
   <si>
+    <t xml:space="preserve">MS_063</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_064</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_065</t>
   </si>
   <si>
@@ -101,12 +125,39 @@
     <t xml:space="preserve">MS_072</t>
   </si>
   <si>
+    <t xml:space="preserve">MS_085</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_087</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_089</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_090</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_091</t>
   </si>
   <si>
     <t xml:space="preserve">MS_092</t>
   </si>
   <si>
+    <t xml:space="preserve">MS_093</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_095</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_097</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_099</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_100</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_101</t>
   </si>
   <si>
@@ -158,6 +209,9 @@
     <t xml:space="preserve">MS_137</t>
   </si>
   <si>
+    <t xml:space="preserve">MS_138</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_141</t>
   </si>
   <si>
@@ -173,6 +227,9 @@
     <t xml:space="preserve">MS_146</t>
   </si>
   <si>
+    <t xml:space="preserve">MS_153</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_155</t>
   </si>
   <si>
@@ -203,6 +260,9 @@
     <t xml:space="preserve">MS_166</t>
   </si>
   <si>
+    <t xml:space="preserve">MS_168</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_169</t>
   </si>
   <si>
@@ -224,6 +284,9 @@
     <t xml:space="preserve">MS_264</t>
   </si>
   <si>
+    <t xml:space="preserve">MS_265</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_266</t>
   </si>
   <si>
@@ -233,6 +296,9 @@
     <t xml:space="preserve">MS_268</t>
   </si>
   <si>
+    <t xml:space="preserve">MS_269</t>
+  </si>
+  <si>
     <t xml:space="preserve">MS_271</t>
   </si>
   <si>
@@ -242,22 +308,34 @@
     <t xml:space="preserve">MS_273</t>
   </si>
   <si>
+    <t xml:space="preserve">Cluster_10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cluster_11</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cluster_113</t>
   </si>
   <si>
+    <t xml:space="preserve">Cluster_14</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cluster_16</t>
   </si>
   <si>
+    <t xml:space="preserve">Cluster_17</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cluster_20</t>
   </si>
   <si>
+    <t xml:space="preserve">Cluster_23</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cluster_31</t>
   </si>
   <si>
     <t xml:space="preserve">Cluster_337</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cluster_34</t>
   </si>
   <si>
     <t xml:space="preserve">Cluster_5</t>
@@ -833,19 +911,85 @@
       <c r="BX1" t="s">
         <v>75</v>
       </c>
+      <c r="BY1" t="s">
+        <v>76</v>
+      </c>
+      <c r="BZ1" t="s">
+        <v>77</v>
+      </c>
+      <c r="CA1" t="s">
+        <v>78</v>
+      </c>
+      <c r="CB1" t="s">
+        <v>79</v>
+      </c>
+      <c r="CC1" t="s">
+        <v>80</v>
+      </c>
+      <c r="CD1" t="s">
+        <v>81</v>
+      </c>
+      <c r="CE1" t="s">
+        <v>82</v>
+      </c>
+      <c r="CF1" t="s">
+        <v>83</v>
+      </c>
+      <c r="CG1" t="s">
+        <v>84</v>
+      </c>
+      <c r="CH1" t="s">
+        <v>85</v>
+      </c>
+      <c r="CI1" t="s">
+        <v>86</v>
+      </c>
+      <c r="CJ1" t="s">
+        <v>87</v>
+      </c>
+      <c r="CK1" t="s">
+        <v>88</v>
+      </c>
+      <c r="CL1" t="s">
+        <v>89</v>
+      </c>
+      <c r="CM1" t="s">
+        <v>90</v>
+      </c>
+      <c r="CN1" t="s">
+        <v>91</v>
+      </c>
+      <c r="CO1" t="s">
+        <v>92</v>
+      </c>
+      <c r="CP1" t="s">
+        <v>93</v>
+      </c>
+      <c r="CQ1" t="s">
+        <v>94</v>
+      </c>
+      <c r="CR1" t="s">
+        <v>95</v>
+      </c>
+      <c r="CS1" t="s">
+        <v>96</v>
+      </c>
+      <c r="CT1" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="B2" t="n">
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>2816</v>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>1863</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -854,7 +998,7 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -863,25 +1007,25 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>822</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>2809</v>
       </c>
       <c r="M2" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="N2" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="O2" t="n">
-        <v>0</v>
+        <v>619</v>
       </c>
       <c r="P2" t="n">
-        <v>0</v>
+        <v>2810</v>
       </c>
       <c r="Q2" t="n">
         <v>0</v>
@@ -947,13 +1091,13 @@
         <v>0</v>
       </c>
       <c r="AL2" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="AM2" t="n">
-        <v>0</v>
+        <v>861</v>
       </c>
       <c r="AN2" t="n">
-        <v>0</v>
+        <v>254</v>
       </c>
       <c r="AO2" t="n">
         <v>0</v>
@@ -965,13 +1109,13 @@
         <v>0</v>
       </c>
       <c r="AR2" t="n">
-        <v>0</v>
+        <v>1346</v>
       </c>
       <c r="AS2" t="n">
-        <v>0</v>
+        <v>723</v>
       </c>
       <c r="AT2" t="n">
-        <v>0</v>
+        <v>2593</v>
       </c>
       <c r="AU2" t="n">
         <v>0</v>
@@ -1061,27 +1205,93 @@
         <v>0</v>
       </c>
       <c r="BX2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL2" t="n">
+        <v>1694</v>
+      </c>
+      <c r="CM2" t="n">
+        <v>1590</v>
+      </c>
+      <c r="CN2" t="n">
+        <v>1190</v>
+      </c>
+      <c r="CO2" t="n">
+        <v>30</v>
+      </c>
+      <c r="CP2" t="n">
+        <v>83</v>
+      </c>
+      <c r="CQ2" t="n">
+        <v>2753</v>
+      </c>
+      <c r="CR2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT2" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>77</v>
+        <v>99</v>
       </c>
       <c r="B3" t="n">
         <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>231</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>258</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -1123,7 +1333,7 @@
         <v>0</v>
       </c>
       <c r="T3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U3" t="n">
         <v>0</v>
@@ -1132,16 +1342,16 @@
         <v>0</v>
       </c>
       <c r="W3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="X3" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="Y3" t="n">
-        <v>24</v>
+        <v>183</v>
       </c>
       <c r="Z3" t="n">
-        <v>26</v>
+        <v>227</v>
       </c>
       <c r="AA3" t="n">
         <v>0</v>
@@ -1162,16 +1372,16 @@
         <v>0</v>
       </c>
       <c r="AG3" t="n">
-        <v>0</v>
+        <v>79</v>
       </c>
       <c r="AH3" t="n">
-        <v>0</v>
+        <v>82</v>
       </c>
       <c r="AI3" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="AJ3" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="AK3" t="n">
         <v>0</v>
@@ -1183,10 +1393,10 @@
         <v>0</v>
       </c>
       <c r="AN3" t="n">
-        <v>0</v>
+        <v>1412</v>
       </c>
       <c r="AO3" t="n">
-        <v>0</v>
+        <v>2832</v>
       </c>
       <c r="AP3" t="n">
         <v>0</v>
@@ -1195,7 +1405,7 @@
         <v>0</v>
       </c>
       <c r="AR3" t="n">
-        <v>0</v>
+        <v>97</v>
       </c>
       <c r="AS3" t="n">
         <v>0</v>
@@ -1204,16 +1414,16 @@
         <v>0</v>
       </c>
       <c r="AU3" t="n">
-        <v>0</v>
+        <v>1925</v>
       </c>
       <c r="AV3" t="n">
-        <v>0</v>
+        <v>1639</v>
       </c>
       <c r="AW3" t="n">
-        <v>0</v>
+        <v>567</v>
       </c>
       <c r="AX3" t="n">
-        <v>0</v>
+        <v>824</v>
       </c>
       <c r="AY3" t="n">
         <v>0</v>
@@ -1225,13 +1435,13 @@
         <v>0</v>
       </c>
       <c r="BB3" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="BC3" t="n">
         <v>0</v>
       </c>
       <c r="BD3" t="n">
-        <v>0</v>
+        <v>784</v>
       </c>
       <c r="BE3" t="n">
         <v>0</v>
@@ -1261,7 +1471,7 @@
         <v>0</v>
       </c>
       <c r="BN3" t="n">
-        <v>0</v>
+        <v>2730</v>
       </c>
       <c r="BO3" t="n">
         <v>0</v>
@@ -1273,13 +1483,13 @@
         <v>0</v>
       </c>
       <c r="BR3" t="n">
-        <v>0</v>
+        <v>179</v>
       </c>
       <c r="BS3" t="n">
         <v>0</v>
       </c>
       <c r="BT3" t="n">
-        <v>0</v>
+        <v>2126</v>
       </c>
       <c r="BU3" t="n">
         <v>0</v>
@@ -1291,12 +1501,78 @@
         <v>0</v>
       </c>
       <c r="BX3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE3" t="n">
+        <v>477</v>
+      </c>
+      <c r="CF3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR3" t="n">
+        <v>15</v>
+      </c>
+      <c r="CS3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>78</v>
+        <v>100</v>
       </c>
       <c r="B4" t="n">
         <v>0</v>
@@ -1311,7 +1587,7 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -1320,13 +1596,13 @@
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -1350,37 +1626,37 @@
         <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>149</v>
+        <v>0</v>
       </c>
       <c r="T4" t="n">
-        <v>153</v>
+        <v>0</v>
       </c>
       <c r="U4" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="V4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y4" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="Z4" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="AA4" t="n">
-        <v>128</v>
+        <v>0</v>
       </c>
       <c r="AB4" t="n">
-        <v>116</v>
+        <v>0</v>
       </c>
       <c r="AC4" t="n">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="AD4" t="n">
         <v>0</v>
@@ -1389,16 +1665,16 @@
         <v>0</v>
       </c>
       <c r="AF4" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="AG4" t="n">
-        <v>175</v>
+        <v>0</v>
       </c>
       <c r="AH4" t="n">
         <v>0</v>
       </c>
       <c r="AI4" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="AJ4" t="n">
         <v>0</v>
@@ -1410,10 +1686,10 @@
         <v>0</v>
       </c>
       <c r="AM4" t="n">
-        <v>101</v>
+        <v>0</v>
       </c>
       <c r="AN4" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="AO4" t="n">
         <v>0</v>
@@ -1440,13 +1716,13 @@
         <v>0</v>
       </c>
       <c r="AW4" t="n">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="AX4" t="n">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="AY4" t="n">
-        <v>79</v>
+        <v>0</v>
       </c>
       <c r="AZ4" t="n">
         <v>0</v>
@@ -1464,7 +1740,7 @@
         <v>0</v>
       </c>
       <c r="BE4" t="n">
-        <v>102</v>
+        <v>0</v>
       </c>
       <c r="BF4" t="n">
         <v>0</v>
@@ -1482,16 +1758,16 @@
         <v>0</v>
       </c>
       <c r="BK4" t="n">
-        <v>76</v>
+        <v>0</v>
       </c>
       <c r="BL4" t="n">
-        <v>116</v>
+        <v>0</v>
       </c>
       <c r="BM4" t="n">
         <v>0</v>
       </c>
       <c r="BN4" t="n">
-        <v>71</v>
+        <v>0</v>
       </c>
       <c r="BO4" t="n">
         <v>0</v>
@@ -1512,30 +1788,96 @@
         <v>0</v>
       </c>
       <c r="BU4" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="BV4" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="BW4" t="n">
         <v>0</v>
       </c>
       <c r="BX4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>79</v>
+        <v>101</v>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>1856</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>83</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -1568,28 +1910,28 @@
         <v>0</v>
       </c>
       <c r="O5" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="P5" t="n">
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="R5" t="n">
-        <v>0</v>
+        <v>363</v>
       </c>
       <c r="S5" t="n">
-        <v>0</v>
+        <v>393</v>
       </c>
       <c r="T5" t="n">
         <v>0</v>
       </c>
       <c r="U5" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="V5" t="n">
-        <v>0</v>
+        <v>401</v>
       </c>
       <c r="W5" t="n">
         <v>0</v>
@@ -1610,10 +1952,10 @@
         <v>0</v>
       </c>
       <c r="AC5" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="AD5" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="AE5" t="n">
         <v>0</v>
@@ -1622,7 +1964,7 @@
         <v>0</v>
       </c>
       <c r="AG5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH5" t="n">
         <v>0</v>
@@ -1658,7 +2000,7 @@
         <v>0</v>
       </c>
       <c r="AS5" t="n">
-        <v>0</v>
+        <v>2250</v>
       </c>
       <c r="AT5" t="n">
         <v>0</v>
@@ -1670,7 +2012,7 @@
         <v>0</v>
       </c>
       <c r="AW5" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="AX5" t="n">
         <v>0</v>
@@ -1751,33 +2093,99 @@
         <v>0</v>
       </c>
       <c r="BX5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ5" t="n">
+        <v>43</v>
+      </c>
+      <c r="CK5" t="n">
+        <v>167</v>
+      </c>
+      <c r="CL5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN5" t="n">
+        <v>94</v>
+      </c>
+      <c r="CO5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>80</v>
+        <v>102</v>
       </c>
       <c r="B6" t="n">
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F6" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>235</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>261</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -1798,34 +2206,34 @@
         <v>0</v>
       </c>
       <c r="O6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P6" t="n">
         <v>0</v>
       </c>
       <c r="Q6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" t="n">
         <v>1</v>
-      </c>
-      <c r="R6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T6" t="n">
-        <v>0</v>
-      </c>
-      <c r="U6" t="n">
-        <v>1</v>
-      </c>
-      <c r="V6" t="n">
-        <v>0</v>
-      </c>
-      <c r="W6" t="n">
-        <v>0</v>
-      </c>
-      <c r="X6" t="n">
-        <v>0</v>
       </c>
       <c r="Y6" t="n">
         <v>0</v>
@@ -1846,16 +2254,16 @@
         <v>0</v>
       </c>
       <c r="AE6" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="AF6" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="AG6" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="AH6" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="AI6" t="n">
         <v>0</v>
@@ -1873,10 +2281,10 @@
         <v>0</v>
       </c>
       <c r="AN6" t="n">
-        <v>0</v>
+        <v>1260</v>
       </c>
       <c r="AO6" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="AP6" t="n">
         <v>0</v>
@@ -1981,12 +2389,78 @@
         <v>0</v>
       </c>
       <c r="BX6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>81</v>
+        <v>103</v>
       </c>
       <c r="B7" t="n">
         <v>0</v>
@@ -1998,10 +2472,10 @@
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -2046,7 +2520,7 @@
         <v>0</v>
       </c>
       <c r="U7" t="n">
-        <v>0</v>
+        <v>118</v>
       </c>
       <c r="V7" t="n">
         <v>0</v>
@@ -2094,7 +2568,7 @@
         <v>0</v>
       </c>
       <c r="AK7" t="n">
-        <v>0</v>
+        <v>237</v>
       </c>
       <c r="AL7" t="n">
         <v>0</v>
@@ -2115,7 +2589,7 @@
         <v>0</v>
       </c>
       <c r="AR7" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="AS7" t="n">
         <v>0</v>
@@ -2160,10 +2634,10 @@
         <v>0</v>
       </c>
       <c r="BG7" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="BH7" t="n">
-        <v>0</v>
+        <v>482</v>
       </c>
       <c r="BI7" t="n">
         <v>0</v>
@@ -2212,119 +2686,185 @@
       </c>
       <c r="BX7" t="n">
         <v>0</v>
+      </c>
+      <c r="BY7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI7" t="n">
+        <v>961</v>
+      </c>
+      <c r="CJ7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT7" t="n">
+        <v>37</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>82</v>
+        <v>104</v>
       </c>
       <c r="B8" t="n">
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>2942</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>2876</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>2756</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>2559</v>
+        <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>2959</v>
+        <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>2606</v>
+        <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>2808</v>
+        <v>0</v>
       </c>
       <c r="M8" t="n">
-        <v>2572</v>
+        <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>519</v>
+        <v>0</v>
       </c>
       <c r="O8" t="n">
-        <v>2727</v>
+        <v>26</v>
       </c>
       <c r="P8" t="n">
-        <v>2564</v>
+        <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>2602</v>
+        <v>0</v>
       </c>
       <c r="R8" t="n">
-        <v>2714</v>
+        <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>1830</v>
+        <v>0</v>
       </c>
       <c r="T8" t="n">
-        <v>1859</v>
+        <v>0</v>
       </c>
       <c r="U8" t="n">
-        <v>1831</v>
+        <v>0</v>
       </c>
       <c r="V8" t="n">
-        <v>1800</v>
+        <v>0</v>
       </c>
       <c r="W8" t="n">
-        <v>1745</v>
+        <v>0</v>
       </c>
       <c r="X8" t="n">
-        <v>1884</v>
+        <v>0</v>
       </c>
       <c r="Y8" t="n">
-        <v>1312</v>
+        <v>155</v>
       </c>
       <c r="Z8" t="n">
-        <v>1763</v>
+        <v>147</v>
       </c>
       <c r="AA8" t="n">
-        <v>1016</v>
+        <v>6</v>
       </c>
       <c r="AB8" t="n">
-        <v>979</v>
+        <v>7</v>
       </c>
       <c r="AC8" t="n">
-        <v>444</v>
+        <v>0</v>
       </c>
       <c r="AD8" t="n">
         <v>0</v>
       </c>
       <c r="AE8" t="n">
-        <v>776</v>
+        <v>4</v>
       </c>
       <c r="AF8" t="n">
         <v>0</v>
       </c>
       <c r="AG8" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="AH8" t="n">
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="AI8" t="n">
-        <v>0</v>
+        <v>115</v>
       </c>
       <c r="AJ8" t="n">
-        <v>706</v>
+        <v>123</v>
       </c>
       <c r="AK8" t="n">
-        <v>320</v>
+        <v>57</v>
       </c>
       <c r="AL8" t="n">
         <v>0</v>
@@ -2333,16 +2873,16 @@
         <v>0</v>
       </c>
       <c r="AN8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AO8" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="AP8" t="n">
         <v>0</v>
       </c>
       <c r="AQ8" t="n">
-        <v>789</v>
+        <v>0</v>
       </c>
       <c r="AR8" t="n">
         <v>0</v>
@@ -2351,25 +2891,25 @@
         <v>0</v>
       </c>
       <c r="AT8" t="n">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="AU8" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="AV8" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="AW8" t="n">
-        <v>235</v>
+        <v>58</v>
       </c>
       <c r="AX8" t="n">
-        <v>0</v>
+        <v>124</v>
       </c>
       <c r="AY8" t="n">
         <v>0</v>
       </c>
       <c r="AZ8" t="n">
-        <v>0</v>
+        <v>106</v>
       </c>
       <c r="BA8" t="n">
         <v>0</v>
@@ -2381,10 +2921,10 @@
         <v>0</v>
       </c>
       <c r="BD8" t="n">
-        <v>0</v>
+        <v>83</v>
       </c>
       <c r="BE8" t="n">
-        <v>0</v>
+        <v>77</v>
       </c>
       <c r="BF8" t="n">
         <v>0</v>
@@ -2414,39 +2954,105 @@
         <v>0</v>
       </c>
       <c r="BO8" t="n">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="BP8" t="n">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="BQ8" t="n">
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="BR8" t="n">
         <v>0</v>
       </c>
       <c r="BS8" t="n">
-        <v>1230</v>
+        <v>0</v>
       </c>
       <c r="BT8" t="n">
-        <v>3000</v>
+        <v>50</v>
       </c>
       <c r="BU8" t="n">
-        <v>2238</v>
+        <v>0</v>
       </c>
       <c r="BV8" t="n">
-        <v>2562</v>
+        <v>0</v>
       </c>
       <c r="BW8" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="BX8" t="n">
-        <v>2559</v>
+        <v>132</v>
+      </c>
+      <c r="BY8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD8" t="n">
+        <v>78</v>
+      </c>
+      <c r="CE8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF8" t="n">
+        <v>111</v>
+      </c>
+      <c r="CG8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH8" t="n">
+        <v>92</v>
+      </c>
+      <c r="CI8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP8" t="n">
+        <v>35</v>
+      </c>
+      <c r="CQ8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR8" t="n">
+        <v>2</v>
+      </c>
+      <c r="CS8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>83</v>
+        <v>105</v>
       </c>
       <c r="B9" t="n">
         <v>0</v>
@@ -2461,7 +3067,7 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>151</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -2653,10 +3259,10 @@
         <v>0</v>
       </c>
       <c r="BR9" t="n">
-        <v>0</v>
+        <v>196</v>
       </c>
       <c r="BS9" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="BT9" t="n">
         <v>0</v>
@@ -2671,12 +3277,78 @@
         <v>0</v>
       </c>
       <c r="BX9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>84</v>
+        <v>106</v>
       </c>
       <c r="B10" t="n">
         <v>0</v>
@@ -2691,7 +3363,7 @@
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -2706,7 +3378,7 @@
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>217</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
@@ -2718,163 +3390,163 @@
         <v>0</v>
       </c>
       <c r="O10" t="n">
-        <v>268</v>
+        <v>0</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>397</v>
+        <v>0</v>
       </c>
       <c r="R10" t="n">
-        <v>286</v>
+        <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>58</v>
+        <v>0</v>
       </c>
       <c r="T10" t="n">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="U10" t="n">
-        <v>1161</v>
+        <v>0</v>
       </c>
       <c r="V10" t="n">
-        <v>1194</v>
+        <v>0</v>
       </c>
       <c r="W10" t="n">
-        <v>1245</v>
+        <v>0</v>
       </c>
       <c r="X10" t="n">
-        <v>1108</v>
+        <v>0</v>
       </c>
       <c r="Y10" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="Z10" t="n">
         <v>0</v>
       </c>
       <c r="AA10" t="n">
-        <v>1581</v>
+        <v>0</v>
       </c>
       <c r="AB10" t="n">
-        <v>1605</v>
+        <v>0</v>
       </c>
       <c r="AC10" t="n">
-        <v>2394</v>
+        <v>0</v>
       </c>
       <c r="AD10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="AE10" t="n">
-        <v>2224</v>
+        <v>0</v>
       </c>
       <c r="AF10" t="n">
-        <v>669</v>
+        <v>1</v>
       </c>
       <c r="AG10" t="n">
         <v>0</v>
       </c>
       <c r="AH10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="AI10" t="n">
-        <v>2404</v>
+        <v>0</v>
       </c>
       <c r="AJ10" t="n">
-        <v>2294</v>
+        <v>0</v>
       </c>
       <c r="AK10" t="n">
-        <v>2680</v>
+        <v>0</v>
       </c>
       <c r="AL10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="AM10" t="n">
-        <v>1821</v>
+        <v>0</v>
       </c>
       <c r="AN10" t="n">
-        <v>676</v>
+        <v>0</v>
       </c>
       <c r="AO10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="AP10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="AQ10" t="n">
-        <v>2211</v>
+        <v>0</v>
       </c>
       <c r="AR10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="AS10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="AT10" t="n">
-        <v>2961</v>
+        <v>0</v>
       </c>
       <c r="AU10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="AV10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="AW10" t="n">
-        <v>2530</v>
+        <v>0</v>
       </c>
       <c r="AX10" t="n">
-        <v>676</v>
+        <v>0</v>
       </c>
       <c r="AY10" t="n">
-        <v>483</v>
+        <v>0</v>
       </c>
       <c r="AZ10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="BA10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="BB10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="BC10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="BD10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="BE10" t="n">
-        <v>900</v>
+        <v>0</v>
       </c>
       <c r="BF10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="BG10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="BH10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="BI10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="BJ10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="BK10" t="n">
-        <v>798</v>
+        <v>0</v>
       </c>
       <c r="BL10" t="n">
-        <v>1894</v>
+        <v>0</v>
       </c>
       <c r="BM10" t="n">
-        <v>2870</v>
+        <v>0</v>
       </c>
       <c r="BN10" t="n">
-        <v>2640</v>
+        <v>0</v>
       </c>
       <c r="BO10" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="BP10" t="n">
         <v>0</v>
@@ -2892,24 +3564,90 @@
         <v>0</v>
       </c>
       <c r="BU10" t="n">
-        <v>517</v>
+        <v>0</v>
       </c>
       <c r="BV10" t="n">
-        <v>401</v>
+        <v>0</v>
       </c>
       <c r="BW10" t="n">
         <v>0</v>
       </c>
       <c r="BX10" t="n">
-        <v>404</v>
+        <v>0</v>
+      </c>
+      <c r="BY10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>85</v>
+        <v>107</v>
       </c>
       <c r="B11" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="C11" t="n">
         <v>0</v>
@@ -2918,16 +3656,16 @@
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
@@ -2936,22 +3674,22 @@
         <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>146</v>
+        <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>192</v>
+        <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>428</v>
+        <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>2481</v>
+        <v>0</v>
       </c>
       <c r="O11" t="n">
         <v>0</v>
       </c>
       <c r="P11" t="n">
-        <v>436</v>
+        <v>0</v>
       </c>
       <c r="Q11" t="n">
         <v>0</v>
@@ -2960,10 +3698,10 @@
         <v>0</v>
       </c>
       <c r="S11" t="n">
-        <v>963</v>
+        <v>0</v>
       </c>
       <c r="T11" t="n">
-        <v>867</v>
+        <v>5</v>
       </c>
       <c r="U11" t="n">
         <v>0</v>
@@ -2972,25 +3710,25 @@
         <v>0</v>
       </c>
       <c r="W11" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="X11" t="n">
         <v>0</v>
       </c>
       <c r="Y11" t="n">
-        <v>1630</v>
+        <v>0</v>
       </c>
       <c r="Z11" t="n">
-        <v>1161</v>
+        <v>0</v>
       </c>
       <c r="AA11" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="AB11" t="n">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="AC11" t="n">
-        <v>92</v>
+        <v>0</v>
       </c>
       <c r="AD11" t="n">
         <v>0</v>
@@ -2999,16 +3737,16 @@
         <v>0</v>
       </c>
       <c r="AF11" t="n">
-        <v>494</v>
+        <v>0</v>
       </c>
       <c r="AG11" t="n">
-        <v>234</v>
+        <v>0</v>
       </c>
       <c r="AH11" t="n">
         <v>0</v>
       </c>
       <c r="AI11" t="n">
-        <v>501</v>
+        <v>0</v>
       </c>
       <c r="AJ11" t="n">
         <v>0</v>
@@ -3023,7 +3761,7 @@
         <v>0</v>
       </c>
       <c r="AN11" t="n">
-        <v>197</v>
+        <v>0</v>
       </c>
       <c r="AO11" t="n">
         <v>0</v>
@@ -3074,7 +3812,7 @@
         <v>0</v>
       </c>
       <c r="BE11" t="n">
-        <v>1998</v>
+        <v>0</v>
       </c>
       <c r="BF11" t="n">
         <v>0</v>
@@ -3107,22 +3845,22 @@
         <v>0</v>
       </c>
       <c r="BP11" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="BQ11" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="BR11" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="BS11" t="n">
-        <v>1770</v>
+        <v>0</v>
       </c>
       <c r="BT11" t="n">
         <v>0</v>
       </c>
       <c r="BU11" t="n">
-        <v>195</v>
+        <v>0</v>
       </c>
       <c r="BV11" t="n">
         <v>0</v>
@@ -3131,12 +3869,78 @@
         <v>0</v>
       </c>
       <c r="BX11" t="n">
-        <v>37</v>
+        <v>0</v>
+      </c>
+      <c r="BY11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>86</v>
+        <v>108</v>
       </c>
       <c r="B12" t="n">
         <v>0</v>
@@ -3148,25 +3952,25 @@
         <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>2950</v>
       </c>
       <c r="F12" t="n">
-        <v>2</v>
+        <v>2891</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>2765</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>2560</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>2962</v>
       </c>
       <c r="J12" t="n">
-        <v>0</v>
+        <v>2178</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>2938</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -3175,49 +3979,49 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>0</v>
+        <v>2929</v>
       </c>
       <c r="O12" t="n">
-        <v>0</v>
+        <v>2021</v>
       </c>
       <c r="P12" t="n">
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>0</v>
+        <v>2802</v>
       </c>
       <c r="R12" t="n">
-        <v>0</v>
+        <v>2238</v>
       </c>
       <c r="S12" t="n">
-        <v>0</v>
+        <v>501</v>
       </c>
       <c r="T12" t="n">
-        <v>0</v>
+        <v>2708</v>
       </c>
       <c r="U12" t="n">
-        <v>0</v>
+        <v>2744</v>
       </c>
       <c r="V12" t="n">
-        <v>0</v>
+        <v>2197</v>
       </c>
       <c r="W12" t="n">
-        <v>0</v>
+        <v>2591</v>
       </c>
       <c r="X12" t="n">
-        <v>0</v>
+        <v>2717</v>
       </c>
       <c r="Y12" t="n">
-        <v>0</v>
+        <v>1674</v>
       </c>
       <c r="Z12" t="n">
-        <v>0</v>
+        <v>1711</v>
       </c>
       <c r="AA12" t="n">
-        <v>0</v>
+        <v>1843</v>
       </c>
       <c r="AB12" t="n">
-        <v>0</v>
+        <v>1851</v>
       </c>
       <c r="AC12" t="n">
         <v>0</v>
@@ -3226,31 +4030,31 @@
         <v>0</v>
       </c>
       <c r="AE12" t="n">
-        <v>0</v>
+        <v>1763</v>
       </c>
       <c r="AF12" t="n">
-        <v>0</v>
+        <v>1910</v>
       </c>
       <c r="AG12" t="n">
-        <v>0</v>
+        <v>1301</v>
       </c>
       <c r="AH12" t="n">
-        <v>0</v>
+        <v>1772</v>
       </c>
       <c r="AI12" t="n">
-        <v>0</v>
+        <v>1028</v>
       </c>
       <c r="AJ12" t="n">
-        <v>0</v>
+        <v>983</v>
       </c>
       <c r="AK12" t="n">
-        <v>0</v>
+        <v>457</v>
       </c>
       <c r="AL12" t="n">
         <v>0</v>
       </c>
       <c r="AM12" t="n">
-        <v>0</v>
+        <v>2139</v>
       </c>
       <c r="AN12" t="n">
         <v>0</v>
@@ -3262,22 +4066,22 @@
         <v>0</v>
       </c>
       <c r="AQ12" t="n">
-        <v>0</v>
+        <v>763</v>
       </c>
       <c r="AR12" t="n">
-        <v>0</v>
+        <v>1015</v>
       </c>
       <c r="AS12" t="n">
         <v>0</v>
       </c>
       <c r="AT12" t="n">
-        <v>0</v>
+        <v>98</v>
       </c>
       <c r="AU12" t="n">
-        <v>0</v>
+        <v>746</v>
       </c>
       <c r="AV12" t="n">
-        <v>0</v>
+        <v>333</v>
       </c>
       <c r="AW12" t="n">
         <v>0</v>
@@ -3292,10 +4096,10 @@
         <v>0</v>
       </c>
       <c r="BA12" t="n">
-        <v>0</v>
+        <v>725</v>
       </c>
       <c r="BB12" t="n">
-        <v>0</v>
+        <v>344</v>
       </c>
       <c r="BC12" t="n">
         <v>0</v>
@@ -3313,7 +4117,7 @@
         <v>0</v>
       </c>
       <c r="BH12" t="n">
-        <v>0</v>
+        <v>678</v>
       </c>
       <c r="BI12" t="n">
         <v>0</v>
@@ -3322,7 +4126,7 @@
         <v>0</v>
       </c>
       <c r="BK12" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="BL12" t="n">
         <v>0</v>
@@ -3334,7 +4138,7 @@
         <v>0</v>
       </c>
       <c r="BO12" t="n">
-        <v>0</v>
+        <v>210</v>
       </c>
       <c r="BP12" t="n">
         <v>0</v>
@@ -3362,11 +4166,77 @@
       </c>
       <c r="BX12" t="n">
         <v>0</v>
+      </c>
+      <c r="BY12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ12" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA12" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB12" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC12" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD12" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE12" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF12" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG12" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH12" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI12" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ12" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK12" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL12" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM12" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN12" t="n">
+        <v>703</v>
+      </c>
+      <c r="CO12" t="n">
+        <v>2970</v>
+      </c>
+      <c r="CP12" t="n">
+        <v>2184</v>
+      </c>
+      <c r="CQ12" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR12" t="n">
+        <v>2569</v>
+      </c>
+      <c r="CS12" t="n">
+        <v>3000</v>
+      </c>
+      <c r="CT12" t="n">
+        <v>2473</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>87</v>
+        <v>109</v>
       </c>
       <c r="B13" t="n">
         <v>0</v>
@@ -3387,7 +4257,7 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>164</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
@@ -3444,153 +4314,1403 @@
         <v>0</v>
       </c>
       <c r="AA13" t="n">
-        <v>220</v>
+        <v>0</v>
       </c>
       <c r="AB13" t="n">
-        <v>241</v>
+        <v>0</v>
       </c>
       <c r="AC13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN13" t="n">
+        <v>5</v>
+      </c>
+      <c r="AO13" t="n">
+        <v>5</v>
+      </c>
+      <c r="AP13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR13" t="n">
+        <v>21</v>
+      </c>
+      <c r="AS13" t="n">
+        <v>27</v>
+      </c>
+      <c r="AT13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU13" t="n">
+        <v>40</v>
+      </c>
+      <c r="AV13" t="n">
+        <v>19</v>
+      </c>
+      <c r="AW13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS13" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>110</v>
+      </c>
+      <c r="B14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" t="n">
+        <v>183</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" t="n">
+        <v>287</v>
+      </c>
+      <c r="U14" t="n">
+        <v>122</v>
+      </c>
+      <c r="V14" t="n">
+        <v>0</v>
+      </c>
+      <c r="W14" t="n">
+        <v>409</v>
+      </c>
+      <c r="X14" t="n">
+        <v>282</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>49</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>81</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>1151</v>
+      </c>
+      <c r="AB14" t="n">
+        <v>1142</v>
+      </c>
+      <c r="AC14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE14" t="n">
+        <v>1221</v>
+      </c>
+      <c r="AF14" t="n">
+        <v>1082</v>
+      </c>
+      <c r="AG14" t="n">
+        <v>8</v>
+      </c>
+      <c r="AH14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI14" t="n">
+        <v>1532</v>
+      </c>
+      <c r="AJ14" t="n">
+        <v>1529</v>
+      </c>
+      <c r="AK14" t="n">
+        <v>2157</v>
+      </c>
+      <c r="AL14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="AQ14" t="n">
+        <v>2237</v>
+      </c>
+      <c r="AR14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT14" t="n">
+        <v>306</v>
+      </c>
+      <c r="AU14" t="n">
+        <v>71</v>
+      </c>
+      <c r="AV14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW14" t="n">
+        <v>522</v>
+      </c>
+      <c r="AX14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="AZ14" t="n">
+        <v>2334</v>
+      </c>
+      <c r="BA14" t="n">
+        <v>2275</v>
+      </c>
+      <c r="BB14" t="n">
+        <v>2615</v>
+      </c>
+      <c r="BC14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="BD14" t="n">
+        <v>1345</v>
+      </c>
+      <c r="BE14" t="n">
+        <v>647</v>
+      </c>
+      <c r="BF14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="BG14" t="n">
+        <v>2976</v>
+      </c>
+      <c r="BH14" t="n">
+        <v>1840</v>
+      </c>
+      <c r="BI14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="BJ14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="BK14" t="n">
+        <v>2954</v>
+      </c>
+      <c r="BL14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="BM14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="BN14" t="n">
+        <v>270</v>
+      </c>
+      <c r="BO14" t="n">
+        <v>2573</v>
+      </c>
+      <c r="BP14" t="n">
+        <v>626</v>
+      </c>
+      <c r="BQ14" t="n">
+        <v>486</v>
+      </c>
+      <c r="BR14" t="n">
+        <v>2625</v>
+      </c>
+      <c r="BS14" t="n">
+        <v>2956</v>
+      </c>
+      <c r="BT14" t="n">
+        <v>651</v>
+      </c>
+      <c r="BU14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="BV14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="BW14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="BX14" t="n">
+        <v>940</v>
+      </c>
+      <c r="BY14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="BZ14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="CA14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="CB14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="CC14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="CD14" t="n">
+        <v>780</v>
+      </c>
+      <c r="CE14" t="n">
+        <v>2523</v>
+      </c>
+      <c r="CF14" t="n">
+        <v>1948</v>
+      </c>
+      <c r="CG14" t="n">
+        <v>2870</v>
+      </c>
+      <c r="CH14" t="n">
+        <v>2636</v>
+      </c>
+      <c r="CI14" t="n">
+        <v>2039</v>
+      </c>
+      <c r="CJ14" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK14" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL14" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM14" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN14" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO14" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP14" t="n">
+        <v>499</v>
+      </c>
+      <c r="CQ14" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR14" t="n">
+        <v>385</v>
+      </c>
+      <c r="CS14" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT14" t="n">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>111</v>
+      </c>
+      <c r="B15" t="n">
+        <v>1144</v>
+      </c>
+      <c r="C15" t="n">
+        <v>184</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1137</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="n">
+        <v>191</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" t="n">
+        <v>130</v>
+      </c>
+      <c r="P15" t="n">
+        <v>190</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>156</v>
+      </c>
+      <c r="R15" t="n">
+        <v>399</v>
+      </c>
+      <c r="S15" t="n">
+        <v>2106</v>
+      </c>
+      <c r="T15" t="n">
+        <v>0</v>
+      </c>
+      <c r="U15" t="n">
+        <v>0</v>
+      </c>
+      <c r="V15" t="n">
+        <v>402</v>
+      </c>
+      <c r="W15" t="n">
+        <v>0</v>
+      </c>
+      <c r="X15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>939</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>833</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE15" t="n">
         <v>1</v>
       </c>
-      <c r="AD13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF13" t="n">
-        <v>1782</v>
-      </c>
-      <c r="AG13" t="n">
-        <v>2591</v>
-      </c>
-      <c r="AH13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM13" t="n">
-        <v>1078</v>
-      </c>
-      <c r="AN13" t="n">
-        <v>2052</v>
-      </c>
-      <c r="AO13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW13" t="n">
-        <v>163</v>
-      </c>
-      <c r="AX13" t="n">
-        <v>2255</v>
-      </c>
-      <c r="AY13" t="n">
-        <v>2438</v>
-      </c>
-      <c r="AZ13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BH13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BI13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BJ13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BK13" t="n">
-        <v>2126</v>
-      </c>
-      <c r="BL13" t="n">
-        <v>990</v>
-      </c>
-      <c r="BM13" t="n">
+      <c r="AF15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG15" t="n">
+        <v>1562</v>
+      </c>
+      <c r="AH15" t="n">
+        <v>1068</v>
+      </c>
+      <c r="AI15" t="n">
+        <v>49</v>
+      </c>
+      <c r="AJ15" t="n">
+        <v>54</v>
+      </c>
+      <c r="AK15" t="n">
+        <v>92</v>
+      </c>
+      <c r="AL15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN15" t="n">
+        <v>65</v>
+      </c>
+      <c r="AO15" t="n">
+        <v>122</v>
+      </c>
+      <c r="AP15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR15" t="n">
+        <v>361</v>
+      </c>
+      <c r="AS15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT15" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU15" t="n">
+        <v>204</v>
+      </c>
+      <c r="AV15" t="n">
+        <v>960</v>
+      </c>
+      <c r="AW15" t="n">
+        <v>410</v>
+      </c>
+      <c r="AX15" t="n">
+        <v>184</v>
+      </c>
+      <c r="AY15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ15" t="n">
+        <v>560</v>
+      </c>
+      <c r="BA15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE15" t="n">
+        <v>205</v>
+      </c>
+      <c r="BF15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT15" t="n">
+        <v>106</v>
+      </c>
+      <c r="BU15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX15" t="n">
+        <v>1928</v>
+      </c>
+      <c r="BY15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ15" t="n">
+        <v>2957</v>
+      </c>
+      <c r="CK15" t="n">
+        <v>2833</v>
+      </c>
+      <c r="CL15" t="n">
+        <v>1306</v>
+      </c>
+      <c r="CM15" t="n">
+        <v>1410</v>
+      </c>
+      <c r="CN15" t="n">
+        <v>1013</v>
+      </c>
+      <c r="CO15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP15" t="n">
+        <v>199</v>
+      </c>
+      <c r="CQ15" t="n">
+        <v>247</v>
+      </c>
+      <c r="CR15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT15" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>112</v>
+      </c>
+      <c r="B16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" t="n">
+        <v>0</v>
+      </c>
+      <c r="T16" t="n">
+        <v>0</v>
+      </c>
+      <c r="U16" t="n">
+        <v>0</v>
+      </c>
+      <c r="V16" t="n">
+        <v>0</v>
+      </c>
+      <c r="W16" t="n">
+        <v>0</v>
+      </c>
+      <c r="X16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>113</v>
+      </c>
+      <c r="B17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" t="n">
+        <v>0</v>
+      </c>
+      <c r="T17" t="n">
+        <v>0</v>
+      </c>
+      <c r="U17" t="n">
+        <v>0</v>
+      </c>
+      <c r="V17" t="n">
+        <v>0</v>
+      </c>
+      <c r="W17" t="n">
+        <v>0</v>
+      </c>
+      <c r="X17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI17" t="n">
+        <v>211</v>
+      </c>
+      <c r="AJ17" t="n">
+        <v>240</v>
+      </c>
+      <c r="AK17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW17" t="n">
+        <v>1417</v>
+      </c>
+      <c r="AX17" t="n">
+        <v>1868</v>
+      </c>
+      <c r="AY17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD17" t="n">
+        <v>788</v>
+      </c>
+      <c r="BE17" t="n">
+        <v>2071</v>
+      </c>
+      <c r="BF17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO17" t="n">
+        <v>145</v>
+      </c>
+      <c r="BP17" t="n">
+        <v>2302</v>
+      </c>
+      <c r="BQ17" t="n">
+        <v>2451</v>
+      </c>
+      <c r="BR17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT17" t="n">
+        <v>67</v>
+      </c>
+      <c r="BU17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD17" t="n">
+        <v>2142</v>
+      </c>
+      <c r="CE17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF17" t="n">
+        <v>941</v>
+      </c>
+      <c r="CG17" t="n">
         <v>130</v>
       </c>
-      <c r="BN13" t="n">
-        <v>289</v>
-      </c>
-      <c r="BO13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BP13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BR13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BS13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BT13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BU13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BV13" t="n">
+      <c r="CH17" t="n">
+        <v>272</v>
+      </c>
+      <c r="CI17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR17" t="n">
         <v>29</v>
       </c>
-      <c r="BW13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BX13" t="n">
+      <c r="CS17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT17" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>